<commit_message>
Lower all ground levels by 25 cm instead of 15 cm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/area2_levels_1114.85.xlsx
+++ b/area2_levels_1114.85.xlsx
@@ -515,19 +515,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1122.261</v>
+        <v>1122.161</v>
       </c>
       <c r="C2" t="n">
-        <v>1121.99</v>
+        <v>1121.89</v>
       </c>
       <c r="D2" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="E2" t="n">
-        <v>1122.71</v>
+        <v>1122.61</v>
       </c>
       <c r="F2" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="G2" t="n">
         <v>1.45</v>
@@ -542,10 +542,10 @@
         <v>355976.049</v>
       </c>
       <c r="K2" t="n">
-        <v>7.411</v>
+        <v>7.311</v>
       </c>
       <c r="L2" t="n">
-        <v>10.78</v>
+        <v>10.64</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -556,19 +556,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="C3" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="D3" t="n">
-        <v>1123.41</v>
+        <v>1123.31</v>
       </c>
       <c r="E3" t="n">
-        <v>1122.75</v>
+        <v>1122.65</v>
       </c>
       <c r="F3" t="n">
-        <v>1122.71</v>
+        <v>1122.61</v>
       </c>
       <c r="G3" t="n">
         <v>2.12</v>
@@ -583,10 +583,10 @@
         <v>355976.049</v>
       </c>
       <c r="K3" t="n">
-        <v>7.88</v>
+        <v>7.78</v>
       </c>
       <c r="L3" t="n">
-        <v>16.74</v>
+        <v>16.53</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -597,19 +597,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1123.192</v>
+        <v>1123.092</v>
       </c>
       <c r="C4" t="n">
-        <v>1123.41</v>
+        <v>1123.31</v>
       </c>
       <c r="D4" t="n">
-        <v>1122.04</v>
+        <v>1121.94</v>
       </c>
       <c r="E4" t="n">
-        <v>1124.57</v>
+        <v>1124.47</v>
       </c>
       <c r="F4" t="n">
-        <v>1122.75</v>
+        <v>1122.65</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>355976.049</v>
       </c>
       <c r="K4" t="n">
-        <v>8.342000000000001</v>
+        <v>8.242000000000001</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -638,19 +638,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1124.859</v>
+        <v>1124.759</v>
       </c>
       <c r="C5" t="n">
-        <v>1122.04</v>
+        <v>1121.94</v>
       </c>
       <c r="D5" t="n">
-        <v>1125.9</v>
+        <v>1125.8</v>
       </c>
       <c r="E5" t="n">
-        <v>1126.92</v>
+        <v>1126.82</v>
       </c>
       <c r="F5" t="n">
-        <v>1124.57</v>
+        <v>1124.47</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
         <v>355976.049</v>
       </c>
       <c r="K5" t="n">
-        <v>10.009</v>
+        <v>9.909000000000001</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -679,19 +679,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1122.419</v>
+        <v>1122.319</v>
       </c>
       <c r="C6" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="D6" t="n">
-        <v>1122.71</v>
+        <v>1122.61</v>
       </c>
       <c r="E6" t="n">
-        <v>1122.93</v>
+        <v>1122.83</v>
       </c>
       <c r="F6" t="n">
-        <v>1121.75</v>
+        <v>1121.65</v>
       </c>
       <c r="G6" t="n">
         <v>5.1</v>
@@ -706,10 +706,10 @@
         <v>355973.049</v>
       </c>
       <c r="K6" t="n">
-        <v>7.569</v>
+        <v>7.469</v>
       </c>
       <c r="L6" t="n">
-        <v>38.58</v>
+        <v>38.07</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -720,19 +720,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1123.178</v>
+        <v>1123.078</v>
       </c>
       <c r="C7" t="n">
-        <v>1122.71</v>
+        <v>1122.61</v>
       </c>
       <c r="D7" t="n">
-        <v>1122.75</v>
+        <v>1122.65</v>
       </c>
       <c r="E7" t="n">
-        <v>1124.33</v>
+        <v>1124.23</v>
       </c>
       <c r="F7" t="n">
-        <v>1122.93</v>
+        <v>1122.83</v>
       </c>
       <c r="G7" t="n">
         <v>8.52</v>
@@ -747,10 +747,10 @@
         <v>355973.049</v>
       </c>
       <c r="K7" t="n">
-        <v>8.327999999999999</v>
+        <v>8.228</v>
       </c>
       <c r="L7" t="n">
-        <v>70.98999999999999</v>
+        <v>70.14</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -761,19 +761,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1124.235</v>
+        <v>1124.135</v>
       </c>
       <c r="C8" t="n">
-        <v>1122.75</v>
+        <v>1122.65</v>
       </c>
       <c r="D8" t="n">
-        <v>1124.57</v>
+        <v>1124.47</v>
       </c>
       <c r="E8" t="n">
-        <v>1125.3</v>
+        <v>1125.2</v>
       </c>
       <c r="F8" t="n">
-        <v>1124.33</v>
+        <v>1124.23</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -788,7 +788,7 @@
         <v>355973.049</v>
       </c>
       <c r="K8" t="n">
-        <v>9.385</v>
+        <v>9.285</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -802,19 +802,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>1126.048</v>
+        <v>1125.948</v>
       </c>
       <c r="C9" t="n">
-        <v>1124.57</v>
+        <v>1124.47</v>
       </c>
       <c r="D9" t="n">
-        <v>1126.92</v>
+        <v>1126.82</v>
       </c>
       <c r="E9" t="n">
-        <v>1127.4</v>
+        <v>1127.3</v>
       </c>
       <c r="F9" t="n">
-        <v>1125.3</v>
+        <v>1125.2</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -829,7 +829,7 @@
         <v>355973.049</v>
       </c>
       <c r="K9" t="n">
-        <v>11.198</v>
+        <v>11.098</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -843,19 +843,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>1122.026</v>
+        <v>1121.926</v>
       </c>
       <c r="C10" t="n">
-        <v>1121.75</v>
+        <v>1121.65</v>
       </c>
       <c r="D10" t="n">
-        <v>1122.93</v>
+        <v>1122.83</v>
       </c>
       <c r="E10" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="F10" t="n">
-        <v>1121.6</v>
+        <v>1121.5</v>
       </c>
       <c r="G10" t="n">
         <v>6.16</v>
@@ -870,10 +870,10 @@
         <v>355970.049</v>
       </c>
       <c r="K10" t="n">
-        <v>7.176</v>
+        <v>7.076</v>
       </c>
       <c r="L10" t="n">
-        <v>44.22</v>
+        <v>43.6</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
@@ -884,19 +884,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>1122.774</v>
+        <v>1122.674</v>
       </c>
       <c r="C11" t="n">
-        <v>1122.93</v>
+        <v>1122.83</v>
       </c>
       <c r="D11" t="n">
-        <v>1124.33</v>
+        <v>1124.23</v>
       </c>
       <c r="E11" t="n">
-        <v>1122.01</v>
+        <v>1121.91</v>
       </c>
       <c r="F11" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="G11" t="n">
         <v>8.52</v>
@@ -911,10 +911,10 @@
         <v>355970.049</v>
       </c>
       <c r="K11" t="n">
-        <v>7.924</v>
+        <v>7.824</v>
       </c>
       <c r="L11" t="n">
-        <v>67.52</v>
+        <v>66.67</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -925,19 +925,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>1123.446</v>
+        <v>1123.346</v>
       </c>
       <c r="C12" t="n">
-        <v>1124.33</v>
+        <v>1124.23</v>
       </c>
       <c r="D12" t="n">
-        <v>1125.3</v>
+        <v>1125.2</v>
       </c>
       <c r="E12" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="F12" t="n">
-        <v>1122.01</v>
+        <v>1121.91</v>
       </c>
       <c r="G12" t="n">
         <v>1.73</v>
@@ -952,10 +952,10 @@
         <v>355970.049</v>
       </c>
       <c r="K12" t="n">
-        <v>8.596</v>
+        <v>8.496</v>
       </c>
       <c r="L12" t="n">
-        <v>14.88</v>
+        <v>14.7</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -966,19 +966,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>1124.654</v>
+        <v>1124.554</v>
       </c>
       <c r="C13" t="n">
-        <v>1125.3</v>
+        <v>1125.2</v>
       </c>
       <c r="D13" t="n">
-        <v>1127.4</v>
+        <v>1127.3</v>
       </c>
       <c r="E13" t="n">
-        <v>1123.76</v>
+        <v>1123.66</v>
       </c>
       <c r="F13" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="G13" t="n">
         <v>1.28</v>
@@ -993,10 +993,10 @@
         <v>355970.049</v>
       </c>
       <c r="K13" t="n">
-        <v>9.804</v>
+        <v>9.704000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>12.59</v>
+        <v>12.46</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
@@ -1007,19 +1007,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>1121.663</v>
+        <v>1121.563</v>
       </c>
       <c r="C14" t="n">
-        <v>1121.6</v>
+        <v>1121.5</v>
       </c>
       <c r="D14" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="E14" t="n">
-        <v>1121.71</v>
+        <v>1121.61</v>
       </c>
       <c r="F14" t="n">
-        <v>1121.5</v>
+        <v>1121.4</v>
       </c>
       <c r="G14" t="n">
         <v>6.06</v>
@@ -1034,10 +1034,10 @@
         <v>355967.049</v>
       </c>
       <c r="K14" t="n">
-        <v>6.813</v>
+        <v>6.713</v>
       </c>
       <c r="L14" t="n">
-        <v>41.26</v>
+        <v>40.65</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
@@ -1048,19 +1048,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>1121.871</v>
+        <v>1121.771</v>
       </c>
       <c r="C15" t="n">
+        <v>1121.73</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1121.91</v>
+      </c>
+      <c r="E15" t="n">
         <v>1121.83</v>
       </c>
-      <c r="D15" t="n">
-        <v>1122.01</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1121.93</v>
-      </c>
       <c r="F15" t="n">
-        <v>1121.71</v>
+        <v>1121.61</v>
       </c>
       <c r="G15" t="n">
         <v>9</v>
@@ -1075,10 +1075,10 @@
         <v>355967.049</v>
       </c>
       <c r="K15" t="n">
-        <v>7.021</v>
+        <v>6.921</v>
       </c>
       <c r="L15" t="n">
-        <v>63.19</v>
+        <v>62.29</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -1089,19 +1089,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>1122.405</v>
+        <v>1122.305</v>
       </c>
       <c r="C16" t="n">
-        <v>1122.01</v>
+        <v>1121.91</v>
       </c>
       <c r="D16" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="E16" t="n">
-        <v>1123.54</v>
+        <v>1123.44</v>
       </c>
       <c r="F16" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="G16" t="n">
         <v>9</v>
@@ -1116,10 +1116,10 @@
         <v>355967.049</v>
       </c>
       <c r="K16" t="n">
-        <v>7.555</v>
+        <v>7.455</v>
       </c>
       <c r="L16" t="n">
-        <v>68</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -1130,19 +1130,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>1124.165</v>
+        <v>1124.065</v>
       </c>
       <c r="C17" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="D17" t="n">
-        <v>1123.76</v>
+        <v>1123.66</v>
       </c>
       <c r="E17" t="n">
-        <v>1127.21</v>
+        <v>1127.11</v>
       </c>
       <c r="F17" t="n">
-        <v>1123.54</v>
+        <v>1123.44</v>
       </c>
       <c r="G17" t="n">
         <v>5.18</v>
@@ -1157,10 +1157,10 @@
         <v>355967.049</v>
       </c>
       <c r="K17" t="n">
-        <v>9.315</v>
+        <v>9.215</v>
       </c>
       <c r="L17" t="n">
-        <v>48.21</v>
+        <v>47.69</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -1171,19 +1171,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>1121.644</v>
+        <v>1121.544</v>
       </c>
       <c r="C18" t="n">
-        <v>1121.5</v>
+        <v>1121.4</v>
       </c>
       <c r="D18" t="n">
-        <v>1121.71</v>
+        <v>1121.61</v>
       </c>
       <c r="E18" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="F18" t="n">
-        <v>1121.59</v>
+        <v>1121.49</v>
       </c>
       <c r="G18" t="n">
         <v>4.67</v>
@@ -1198,10 +1198,10 @@
         <v>355964.049</v>
       </c>
       <c r="K18" t="n">
-        <v>6.794</v>
+        <v>6.694</v>
       </c>
       <c r="L18" t="n">
-        <v>31.76</v>
+        <v>31.29</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -1212,19 +1212,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>1121.843</v>
+        <v>1121.743</v>
       </c>
       <c r="C19" t="n">
-        <v>1121.71</v>
+        <v>1121.61</v>
       </c>
       <c r="D19" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="E19" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="F19" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="G19" t="n">
         <v>9</v>
@@ -1239,10 +1239,10 @@
         <v>355964.049</v>
       </c>
       <c r="K19" t="n">
-        <v>6.993</v>
+        <v>6.893</v>
       </c>
       <c r="L19" t="n">
-        <v>62.94</v>
+        <v>62.04</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
@@ -1253,19 +1253,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>1122.784</v>
+        <v>1122.684</v>
       </c>
       <c r="C20" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="D20" t="n">
-        <v>1123.54</v>
+        <v>1123.44</v>
       </c>
       <c r="E20" t="n">
-        <v>1123.71</v>
+        <v>1123.61</v>
       </c>
       <c r="F20" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="G20" t="n">
         <v>9</v>
@@ -1280,10 +1280,10 @@
         <v>355964.049</v>
       </c>
       <c r="K20" t="n">
-        <v>7.934</v>
+        <v>7.834</v>
       </c>
       <c r="L20" t="n">
-        <v>71.41</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
@@ -1294,19 +1294,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>1125.448</v>
+        <v>1125.348</v>
       </c>
       <c r="C21" t="n">
-        <v>1123.54</v>
+        <v>1123.44</v>
       </c>
       <c r="D21" t="n">
-        <v>1127.21</v>
+        <v>1127.11</v>
       </c>
       <c r="E21" t="n">
-        <v>1127.33</v>
+        <v>1127.23</v>
       </c>
       <c r="F21" t="n">
-        <v>1123.71</v>
+        <v>1123.61</v>
       </c>
       <c r="G21" t="n">
         <v>5.18</v>
@@ -1321,10 +1321,10 @@
         <v>355964.049</v>
       </c>
       <c r="K21" t="n">
-        <v>10.598</v>
+        <v>10.498</v>
       </c>
       <c r="L21" t="n">
-        <v>54.86</v>
+        <v>54.34</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -1335,19 +1335,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>1121.713</v>
+        <v>1121.613</v>
       </c>
       <c r="C22" t="n">
-        <v>1121.59</v>
+        <v>1121.49</v>
       </c>
       <c r="D22" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="E22" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="F22" t="n">
-        <v>1121.67</v>
+        <v>1121.57</v>
       </c>
       <c r="G22" t="n">
         <v>5.75</v>
@@ -1362,10 +1362,10 @@
         <v>355961.049</v>
       </c>
       <c r="K22" t="n">
-        <v>6.863</v>
+        <v>6.763</v>
       </c>
       <c r="L22" t="n">
-        <v>39.46</v>
+        <v>38.88</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
@@ -1376,19 +1376,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>1121.885</v>
+        <v>1121.785</v>
       </c>
       <c r="C23" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="D23" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="E23" t="n">
-        <v>1121.98</v>
+        <v>1121.88</v>
       </c>
       <c r="F23" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="G23" t="n">
         <v>9</v>
@@ -1403,10 +1403,10 @@
         <v>355961.049</v>
       </c>
       <c r="K23" t="n">
-        <v>7.035</v>
+        <v>6.935</v>
       </c>
       <c r="L23" t="n">
-        <v>63.32</v>
+        <v>62.42</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
@@ -1417,19 +1417,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>1122.884</v>
+        <v>1122.784</v>
       </c>
       <c r="C24" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="D24" t="n">
-        <v>1123.71</v>
+        <v>1123.61</v>
       </c>
       <c r="E24" t="n">
-        <v>1123.88</v>
+        <v>1123.78</v>
       </c>
       <c r="F24" t="n">
-        <v>1121.98</v>
+        <v>1121.88</v>
       </c>
       <c r="G24" t="n">
         <v>9</v>
@@ -1444,10 +1444,10 @@
         <v>355961.049</v>
       </c>
       <c r="K24" t="n">
-        <v>8.034000000000001</v>
+        <v>7.934</v>
       </c>
       <c r="L24" t="n">
-        <v>72.31</v>
+        <v>71.41</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
@@ -1458,19 +1458,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>1125.537</v>
+        <v>1125.437</v>
       </c>
       <c r="C25" t="n">
-        <v>1123.71</v>
+        <v>1123.61</v>
       </c>
       <c r="D25" t="n">
-        <v>1127.33</v>
+        <v>1127.23</v>
       </c>
       <c r="E25" t="n">
-        <v>1127.22</v>
+        <v>1127.12</v>
       </c>
       <c r="F25" t="n">
-        <v>1123.88</v>
+        <v>1123.78</v>
       </c>
       <c r="G25" t="n">
         <v>5.18</v>
@@ -1485,10 +1485,10 @@
         <v>355961.049</v>
       </c>
       <c r="K25" t="n">
-        <v>10.687</v>
+        <v>10.587</v>
       </c>
       <c r="L25" t="n">
-        <v>55.33</v>
+        <v>54.82</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
@@ -1499,19 +1499,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>1121.776</v>
+        <v>1121.676</v>
       </c>
       <c r="C26" t="n">
-        <v>1121.67</v>
+        <v>1121.57</v>
       </c>
       <c r="D26" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="E26" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="F26" t="n">
-        <v>1121.74</v>
+        <v>1121.64</v>
       </c>
       <c r="G26" t="n">
         <v>6.82</v>
@@ -1526,10 +1526,10 @@
         <v>355958.049</v>
       </c>
       <c r="K26" t="n">
-        <v>6.926</v>
+        <v>6.826</v>
       </c>
       <c r="L26" t="n">
-        <v>47.26</v>
+        <v>46.58</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
@@ -1540,19 +1540,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>1121.919</v>
+        <v>1121.819</v>
       </c>
       <c r="C27" t="n">
-        <v>1121.83</v>
+        <v>1121.73</v>
       </c>
       <c r="D27" t="n">
-        <v>1121.98</v>
+        <v>1121.88</v>
       </c>
       <c r="E27" t="n">
-        <v>1122</v>
+        <v>1121.9</v>
       </c>
       <c r="F27" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="G27" t="n">
         <v>9</v>
@@ -1567,10 +1567,10 @@
         <v>355958.049</v>
       </c>
       <c r="K27" t="n">
-        <v>7.069</v>
+        <v>6.969</v>
       </c>
       <c r="L27" t="n">
-        <v>63.62</v>
+        <v>62.72</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -1581,19 +1581,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>1122.918</v>
+        <v>1122.818</v>
       </c>
       <c r="C28" t="n">
-        <v>1121.98</v>
+        <v>1121.88</v>
       </c>
       <c r="D28" t="n">
-        <v>1123.88</v>
+        <v>1123.78</v>
       </c>
       <c r="E28" t="n">
-        <v>1123.8</v>
+        <v>1123.7</v>
       </c>
       <c r="F28" t="n">
-        <v>1122</v>
+        <v>1121.9</v>
       </c>
       <c r="G28" t="n">
         <v>9</v>
@@ -1608,10 +1608,10 @@
         <v>355958.049</v>
       </c>
       <c r="K28" t="n">
-        <v>8.068</v>
+        <v>7.968</v>
       </c>
       <c r="L28" t="n">
-        <v>72.61</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="M28" t="n">
         <v>0</v>
@@ -1622,19 +1622,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>1125.534</v>
+        <v>1125.434</v>
       </c>
       <c r="C29" t="n">
-        <v>1123.88</v>
+        <v>1123.78</v>
       </c>
       <c r="D29" t="n">
-        <v>1127.22</v>
+        <v>1127.12</v>
       </c>
       <c r="E29" t="n">
-        <v>1127.23</v>
+        <v>1127.13</v>
       </c>
       <c r="F29" t="n">
-        <v>1123.8</v>
+        <v>1123.7</v>
       </c>
       <c r="G29" t="n">
         <v>5.18</v>
@@ -1649,10 +1649,10 @@
         <v>355958.049</v>
       </c>
       <c r="K29" t="n">
-        <v>10.684</v>
+        <v>10.584</v>
       </c>
       <c r="L29" t="n">
-        <v>55.33</v>
+        <v>54.81</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
@@ -1663,19 +1663,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>1121.709</v>
+        <v>1121.609</v>
       </c>
       <c r="C30" t="n">
-        <v>1121.63</v>
+        <v>1121.53</v>
       </c>
       <c r="D30" t="n">
-        <v>1121.74</v>
+        <v>1121.64</v>
       </c>
       <c r="E30" t="n">
-        <v>1121.8</v>
+        <v>1121.7</v>
       </c>
       <c r="F30" t="n">
-        <v>1121.66</v>
+        <v>1121.56</v>
       </c>
       <c r="G30" t="n">
         <v>1.71</v>
@@ -1690,10 +1690,10 @@
         <v>355955.049</v>
       </c>
       <c r="K30" t="n">
-        <v>6.859</v>
+        <v>6.759</v>
       </c>
       <c r="L30" t="n">
-        <v>11.75</v>
+        <v>11.58</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
@@ -1704,19 +1704,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>1121.834</v>
+        <v>1121.734</v>
       </c>
       <c r="C31" t="n">
-        <v>1121.74</v>
+        <v>1121.64</v>
       </c>
       <c r="D31" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="E31" t="n">
-        <v>1121.92</v>
+        <v>1121.82</v>
       </c>
       <c r="F31" t="n">
-        <v>1121.8</v>
+        <v>1121.7</v>
       </c>
       <c r="G31" t="n">
         <v>8.449999999999999</v>
@@ -1731,10 +1731,10 @@
         <v>355955.049</v>
       </c>
       <c r="K31" t="n">
-        <v>6.984</v>
+        <v>6.884</v>
       </c>
       <c r="L31" t="n">
-        <v>59.02</v>
+        <v>58.18</v>
       </c>
       <c r="M31" t="n">
         <v>0</v>
@@ -1745,19 +1745,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>1121.962</v>
+        <v>1121.862</v>
       </c>
       <c r="C32" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="D32" t="n">
-        <v>1122</v>
+        <v>1121.9</v>
       </c>
       <c r="E32" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="F32" t="n">
-        <v>1121.92</v>
+        <v>1121.82</v>
       </c>
       <c r="G32" t="n">
         <v>9</v>
@@ -1772,10 +1772,10 @@
         <v>355955.049</v>
       </c>
       <c r="K32" t="n">
-        <v>7.112</v>
+        <v>7.012</v>
       </c>
       <c r="L32" t="n">
-        <v>64</v>
+        <v>63.1</v>
       </c>
       <c r="M32" t="n">
         <v>0</v>
@@ -1786,19 +1786,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>1122.832</v>
+        <v>1122.732</v>
       </c>
       <c r="C33" t="n">
-        <v>1122</v>
+        <v>1121.9</v>
       </c>
       <c r="D33" t="n">
-        <v>1123.8</v>
+        <v>1123.7</v>
       </c>
       <c r="E33" t="n">
-        <v>1123.47</v>
+        <v>1123.37</v>
       </c>
       <c r="F33" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="G33" t="n">
         <v>9</v>
@@ -1813,10 +1813,10 @@
         <v>355955.049</v>
       </c>
       <c r="K33" t="n">
-        <v>7.982</v>
+        <v>7.882</v>
       </c>
       <c r="L33" t="n">
-        <v>71.84</v>
+        <v>70.94</v>
       </c>
       <c r="M33" t="n">
         <v>0</v>
@@ -1827,19 +1827,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>1125.08</v>
+        <v>1124.98</v>
       </c>
       <c r="C34" t="n">
-        <v>1123.8</v>
+        <v>1123.7</v>
       </c>
       <c r="D34" t="n">
-        <v>1127.23</v>
+        <v>1127.13</v>
       </c>
       <c r="E34" t="n">
-        <v>1125.82</v>
+        <v>1125.72</v>
       </c>
       <c r="F34" t="n">
-        <v>1123.47</v>
+        <v>1123.37</v>
       </c>
       <c r="G34" t="n">
         <v>5.18</v>
@@ -1854,10 +1854,10 @@
         <v>355955.049</v>
       </c>
       <c r="K34" t="n">
-        <v>10.23</v>
+        <v>10.13</v>
       </c>
       <c r="L34" t="n">
-        <v>52.99</v>
+        <v>52.47</v>
       </c>
       <c r="M34" t="n">
         <v>0</v>
@@ -1868,19 +1868,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>1121.763</v>
+        <v>1121.663</v>
       </c>
       <c r="C35" t="n">
-        <v>1121.66</v>
+        <v>1121.56</v>
       </c>
       <c r="D35" t="n">
-        <v>1121.8</v>
+        <v>1121.7</v>
       </c>
       <c r="E35" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="F35" t="n">
-        <v>1121.73</v>
+        <v>1121.63</v>
       </c>
       <c r="G35" t="n">
         <v>1.28</v>
@@ -1895,10 +1895,10 @@
         <v>355952.049</v>
       </c>
       <c r="K35" t="n">
-        <v>6.913</v>
+        <v>6.813</v>
       </c>
       <c r="L35" t="n">
-        <v>8.83</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M35" t="n">
         <v>0</v>
@@ -1909,19 +1909,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>1121.894</v>
+        <v>1121.794</v>
       </c>
       <c r="C36" t="n">
-        <v>1121.8</v>
+        <v>1121.7</v>
       </c>
       <c r="D36" t="n">
-        <v>1121.92</v>
+        <v>1121.82</v>
       </c>
       <c r="E36" t="n">
-        <v>1121.99</v>
+        <v>1121.89</v>
       </c>
       <c r="F36" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="G36" t="n">
         <v>9</v>
@@ -1936,10 +1936,10 @@
         <v>355952.049</v>
       </c>
       <c r="K36" t="n">
-        <v>7.044</v>
+        <v>6.944</v>
       </c>
       <c r="L36" t="n">
-        <v>63.4</v>
+        <v>62.5</v>
       </c>
       <c r="M36" t="n">
         <v>0</v>
@@ -1950,19 +1950,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>1122.016</v>
+        <v>1121.916</v>
       </c>
       <c r="C37" t="n">
-        <v>1121.92</v>
+        <v>1121.82</v>
       </c>
       <c r="D37" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="E37" t="n">
-        <v>1122.1</v>
+        <v>1122</v>
       </c>
       <c r="F37" t="n">
-        <v>1121.99</v>
+        <v>1121.89</v>
       </c>
       <c r="G37" t="n">
         <v>9</v>
@@ -1977,10 +1977,10 @@
         <v>355952.049</v>
       </c>
       <c r="K37" t="n">
-        <v>7.166</v>
+        <v>7.066</v>
       </c>
       <c r="L37" t="n">
-        <v>64.5</v>
+        <v>63.6</v>
       </c>
       <c r="M37" t="n">
         <v>0</v>
@@ -1991,19 +1991,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>1122.786</v>
+        <v>1122.686</v>
       </c>
       <c r="C38" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="D38" t="n">
-        <v>1123.47</v>
+        <v>1123.37</v>
       </c>
       <c r="E38" t="n">
-        <v>1123.52</v>
+        <v>1123.42</v>
       </c>
       <c r="F38" t="n">
-        <v>1122.1</v>
+        <v>1122</v>
       </c>
       <c r="G38" t="n">
         <v>9</v>
@@ -2018,10 +2018,10 @@
         <v>355952.049</v>
       </c>
       <c r="K38" t="n">
-        <v>7.936</v>
+        <v>7.836</v>
       </c>
       <c r="L38" t="n">
-        <v>71.43000000000001</v>
+        <v>70.53</v>
       </c>
       <c r="M38" t="n">
         <v>0</v>
@@ -2032,19 +2032,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>1124.918</v>
+        <v>1124.818</v>
       </c>
       <c r="C39" t="n">
-        <v>1123.47</v>
+        <v>1123.37</v>
       </c>
       <c r="D39" t="n">
-        <v>1125.82</v>
+        <v>1125.72</v>
       </c>
       <c r="E39" t="n">
-        <v>1126.86</v>
+        <v>1126.76</v>
       </c>
       <c r="F39" t="n">
-        <v>1123.52</v>
+        <v>1123.42</v>
       </c>
       <c r="G39" t="n">
         <v>5.18</v>
@@ -2059,10 +2059,10 @@
         <v>355952.049</v>
       </c>
       <c r="K39" t="n">
-        <v>10.068</v>
+        <v>9.968</v>
       </c>
       <c r="L39" t="n">
-        <v>52.17</v>
+        <v>51.65</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -2073,19 +2073,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>1121.846</v>
+        <v>1121.746</v>
       </c>
       <c r="C40" t="n">
-        <v>1121.73</v>
+        <v>1121.63</v>
       </c>
       <c r="D40" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="E40" t="n">
-        <v>1121.95</v>
+        <v>1121.85</v>
       </c>
       <c r="F40" t="n">
-        <v>1121.85</v>
+        <v>1121.75</v>
       </c>
       <c r="G40" t="n">
         <v>1.75</v>
@@ -2100,10 +2100,10 @@
         <v>355949.049</v>
       </c>
       <c r="K40" t="n">
-        <v>6.996</v>
+        <v>6.896</v>
       </c>
       <c r="L40" t="n">
-        <v>12.23</v>
+        <v>12.05</v>
       </c>
       <c r="M40" t="n">
         <v>0</v>
@@ -2114,19 +2114,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>1121.962</v>
+        <v>1121.862</v>
       </c>
       <c r="C41" t="n">
-        <v>1121.86</v>
+        <v>1121.76</v>
       </c>
       <c r="D41" t="n">
-        <v>1121.99</v>
+        <v>1121.89</v>
       </c>
       <c r="E41" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="F41" t="n">
-        <v>1121.95</v>
+        <v>1121.85</v>
       </c>
       <c r="G41" t="n">
         <v>9</v>
@@ -2141,10 +2141,10 @@
         <v>355949.049</v>
       </c>
       <c r="K41" t="n">
-        <v>7.112</v>
+        <v>7.012</v>
       </c>
       <c r="L41" t="n">
-        <v>64.01000000000001</v>
+        <v>63.11</v>
       </c>
       <c r="M41" t="n">
         <v>0</v>
@@ -2155,19 +2155,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>1122.071</v>
+        <v>1121.971</v>
       </c>
       <c r="C42" t="n">
-        <v>1121.99</v>
+        <v>1121.89</v>
       </c>
       <c r="D42" t="n">
-        <v>1122.1</v>
+        <v>1122</v>
       </c>
       <c r="E42" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="F42" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="G42" t="n">
         <v>9</v>
@@ -2182,10 +2182,10 @@
         <v>355949.049</v>
       </c>
       <c r="K42" t="n">
-        <v>7.221</v>
+        <v>7.121</v>
       </c>
       <c r="L42" t="n">
-        <v>64.98999999999999</v>
+        <v>64.09</v>
       </c>
       <c r="M42" t="n">
         <v>0</v>
@@ -2196,19 +2196,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>1122.79</v>
+        <v>1122.69</v>
       </c>
       <c r="C43" t="n">
-        <v>1122.1</v>
+        <v>1122</v>
       </c>
       <c r="D43" t="n">
-        <v>1123.52</v>
+        <v>1123.42</v>
       </c>
       <c r="E43" t="n">
-        <v>1123.39</v>
+        <v>1123.29</v>
       </c>
       <c r="F43" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="G43" t="n">
         <v>9</v>
@@ -2223,10 +2223,10 @@
         <v>355949.049</v>
       </c>
       <c r="K43" t="n">
-        <v>7.94</v>
+        <v>7.84</v>
       </c>
       <c r="L43" t="n">
-        <v>71.45999999999999</v>
+        <v>70.56</v>
       </c>
       <c r="M43" t="n">
         <v>0</v>
@@ -2237,19 +2237,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>1125.288</v>
+        <v>1125.188</v>
       </c>
       <c r="C44" t="n">
-        <v>1123.52</v>
+        <v>1123.42</v>
       </c>
       <c r="D44" t="n">
-        <v>1126.86</v>
+        <v>1126.76</v>
       </c>
       <c r="E44" t="n">
-        <v>1127.38</v>
+        <v>1127.28</v>
       </c>
       <c r="F44" t="n">
-        <v>1123.39</v>
+        <v>1123.29</v>
       </c>
       <c r="G44" t="n">
         <v>5.18</v>
@@ -2264,10 +2264,10 @@
         <v>355949.049</v>
       </c>
       <c r="K44" t="n">
-        <v>10.438</v>
+        <v>10.338</v>
       </c>
       <c r="L44" t="n">
-        <v>54.1</v>
+        <v>53.58</v>
       </c>
       <c r="M44" t="n">
         <v>0</v>
@@ -2278,19 +2278,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>1121.949</v>
+        <v>1121.849</v>
       </c>
       <c r="C45" t="n">
+        <v>1121.75</v>
+      </c>
+      <c r="D45" t="n">
         <v>1121.85</v>
       </c>
-      <c r="D45" t="n">
+      <c r="E45" t="n">
         <v>1121.95</v>
       </c>
-      <c r="E45" t="n">
-        <v>1122.05</v>
-      </c>
       <c r="F45" t="n">
-        <v>1121.95</v>
+        <v>1121.85</v>
       </c>
       <c r="G45" t="n">
         <v>4.94</v>
@@ -2305,10 +2305,10 @@
         <v>355946.049</v>
       </c>
       <c r="K45" t="n">
-        <v>7.099</v>
+        <v>6.999</v>
       </c>
       <c r="L45" t="n">
-        <v>35.06</v>
+        <v>34.56</v>
       </c>
       <c r="M45" t="n">
         <v>0</v>
@@ -2319,19 +2319,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>1122.079</v>
+        <v>1121.979</v>
       </c>
       <c r="C46" t="n">
+        <v>1121.85</v>
+      </c>
+      <c r="D46" t="n">
         <v>1121.95</v>
       </c>
-      <c r="D46" t="n">
-        <v>1122.05</v>
-      </c>
       <c r="E46" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="F46" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="G46" t="n">
         <v>9</v>
@@ -2346,10 +2346,10 @@
         <v>355946.049</v>
       </c>
       <c r="K46" t="n">
-        <v>7.229</v>
+        <v>7.129</v>
       </c>
       <c r="L46" t="n">
-        <v>65.06999999999999</v>
+        <v>64.17</v>
       </c>
       <c r="M46" t="n">
         <v>0</v>
@@ -2360,19 +2360,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>1122.18</v>
+        <v>1122.08</v>
       </c>
       <c r="C47" t="n">
+        <v>1121.95</v>
+      </c>
+      <c r="D47" t="n">
         <v>1122.05</v>
       </c>
-      <c r="D47" t="n">
-        <v>1122.15</v>
-      </c>
       <c r="E47" t="n">
-        <v>1122.26</v>
+        <v>1122.16</v>
       </c>
       <c r="F47" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="G47" t="n">
         <v>9</v>
@@ -2387,10 +2387,10 @@
         <v>355946.049</v>
       </c>
       <c r="K47" t="n">
-        <v>7.33</v>
+        <v>7.23</v>
       </c>
       <c r="L47" t="n">
-        <v>65.97</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="M47" t="n">
         <v>0</v>
@@ -2401,19 +2401,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>1122.765</v>
+        <v>1122.665</v>
       </c>
       <c r="C48" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="D48" t="n">
-        <v>1123.39</v>
+        <v>1123.29</v>
       </c>
       <c r="E48" t="n">
-        <v>1123.26</v>
+        <v>1123.16</v>
       </c>
       <c r="F48" t="n">
-        <v>1122.26</v>
+        <v>1122.16</v>
       </c>
       <c r="G48" t="n">
         <v>9</v>
@@ -2428,10 +2428,10 @@
         <v>355946.049</v>
       </c>
       <c r="K48" t="n">
-        <v>7.915</v>
+        <v>7.815</v>
       </c>
       <c r="L48" t="n">
-        <v>71.23</v>
+        <v>70.33</v>
       </c>
       <c r="M48" t="n">
         <v>0</v>
@@ -2442,19 +2442,19 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>1125.304</v>
+        <v>1125.204</v>
       </c>
       <c r="C49" t="n">
-        <v>1123.39</v>
+        <v>1123.29</v>
       </c>
       <c r="D49" t="n">
-        <v>1127.38</v>
+        <v>1127.28</v>
       </c>
       <c r="E49" t="n">
-        <v>1127.18</v>
+        <v>1127.08</v>
       </c>
       <c r="F49" t="n">
-        <v>1123.26</v>
+        <v>1123.16</v>
       </c>
       <c r="G49" t="n">
         <v>5.18</v>
@@ -2469,10 +2469,10 @@
         <v>355946.049</v>
       </c>
       <c r="K49" t="n">
-        <v>10.454</v>
+        <v>10.354</v>
       </c>
       <c r="L49" t="n">
-        <v>54.19</v>
+        <v>53.67</v>
       </c>
       <c r="M49" t="n">
         <v>0</v>
@@ -2483,19 +2483,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="C50" t="n">
+        <v>1121.85</v>
+      </c>
+      <c r="D50" t="n">
         <v>1121.95</v>
       </c>
-      <c r="D50" t="n">
-        <v>1122.05</v>
-      </c>
       <c r="E50" t="n">
-        <v>1122.17</v>
+        <v>1122.07</v>
       </c>
       <c r="F50" t="n">
-        <v>1122.03</v>
+        <v>1121.93</v>
       </c>
       <c r="G50" t="n">
         <v>4.41</v>
@@ -2510,10 +2510,10 @@
         <v>355943.049</v>
       </c>
       <c r="K50" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="L50" t="n">
-        <v>31.77</v>
+        <v>31.33</v>
       </c>
       <c r="M50" t="n">
         <v>0</v>
@@ -2524,19 +2524,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>1122.168</v>
+        <v>1122.068</v>
       </c>
       <c r="C51" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="D51" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="E51" t="n">
-        <v>1122.19</v>
+        <v>1122.09</v>
       </c>
       <c r="F51" t="n">
-        <v>1122.17</v>
+        <v>1122.07</v>
       </c>
       <c r="G51" t="n">
         <v>9</v>
@@ -2551,10 +2551,10 @@
         <v>355943.049</v>
       </c>
       <c r="K51" t="n">
-        <v>7.318</v>
+        <v>7.218</v>
       </c>
       <c r="L51" t="n">
-        <v>65.87</v>
+        <v>64.97</v>
       </c>
       <c r="M51" t="n">
         <v>0</v>
@@ -2565,19 +2565,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>1122.241</v>
+        <v>1122.141</v>
       </c>
       <c r="C52" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="D52" t="n">
-        <v>1122.26</v>
+        <v>1122.16</v>
       </c>
       <c r="E52" t="n">
-        <v>1122.25</v>
+        <v>1122.15</v>
       </c>
       <c r="F52" t="n">
-        <v>1122.19</v>
+        <v>1122.09</v>
       </c>
       <c r="G52" t="n">
         <v>9</v>
@@ -2592,10 +2592,10 @@
         <v>355943.049</v>
       </c>
       <c r="K52" t="n">
-        <v>7.391</v>
+        <v>7.291</v>
       </c>
       <c r="L52" t="n">
-        <v>66.52</v>
+        <v>65.62</v>
       </c>
       <c r="M52" t="n">
         <v>0</v>
@@ -2606,19 +2606,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>1122.773</v>
+        <v>1122.673</v>
       </c>
       <c r="C53" t="n">
-        <v>1122.26</v>
+        <v>1122.16</v>
       </c>
       <c r="D53" t="n">
-        <v>1123.26</v>
+        <v>1123.16</v>
       </c>
       <c r="E53" t="n">
-        <v>1123.32</v>
+        <v>1123.22</v>
       </c>
       <c r="F53" t="n">
-        <v>1122.25</v>
+        <v>1122.15</v>
       </c>
       <c r="G53" t="n">
         <v>9</v>
@@ -2633,10 +2633,10 @@
         <v>355943.049</v>
       </c>
       <c r="K53" t="n">
-        <v>7.923</v>
+        <v>7.823</v>
       </c>
       <c r="L53" t="n">
-        <v>71.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="M53" t="n">
         <v>0</v>
@@ -2647,19 +2647,19 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>1125.221</v>
+        <v>1125.121</v>
       </c>
       <c r="C54" t="n">
-        <v>1123.26</v>
+        <v>1123.16</v>
       </c>
       <c r="D54" t="n">
-        <v>1127.18</v>
+        <v>1127.08</v>
       </c>
       <c r="E54" t="n">
-        <v>1127.12</v>
+        <v>1127.02</v>
       </c>
       <c r="F54" t="n">
-        <v>1123.32</v>
+        <v>1123.22</v>
       </c>
       <c r="G54" t="n">
         <v>5.18</v>
@@ -2674,10 +2674,10 @@
         <v>355943.049</v>
       </c>
       <c r="K54" t="n">
-        <v>10.371</v>
+        <v>10.271</v>
       </c>
       <c r="L54" t="n">
-        <v>53.77</v>
+        <v>53.25</v>
       </c>
       <c r="M54" t="n">
         <v>0</v>
@@ -2688,19 +2688,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>1122.129</v>
+        <v>1122.029</v>
       </c>
       <c r="C55" t="n">
-        <v>1122.03</v>
+        <v>1121.93</v>
       </c>
       <c r="D55" t="n">
-        <v>1122.17</v>
+        <v>1122.07</v>
       </c>
       <c r="E55" t="n">
-        <v>1122.21</v>
+        <v>1122.11</v>
       </c>
       <c r="F55" t="n">
-        <v>1122.11</v>
+        <v>1122.01</v>
       </c>
       <c r="G55" t="n">
         <v>4.94</v>
@@ -2715,10 +2715,10 @@
         <v>355940.049</v>
       </c>
       <c r="K55" t="n">
-        <v>7.279</v>
+        <v>7.179</v>
       </c>
       <c r="L55" t="n">
-        <v>35.98</v>
+        <v>35.48</v>
       </c>
       <c r="M55" t="n">
         <v>0</v>
@@ -2729,19 +2729,19 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>1122.123</v>
+        <v>1122.023</v>
       </c>
       <c r="C56" t="n">
-        <v>1122.17</v>
+        <v>1122.07</v>
       </c>
       <c r="D56" t="n">
-        <v>1122.19</v>
+        <v>1122.09</v>
       </c>
       <c r="E56" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="F56" t="n">
-        <v>1122.21</v>
+        <v>1122.11</v>
       </c>
       <c r="G56" t="n">
         <v>9</v>
@@ -2756,10 +2756,10 @@
         <v>355940.049</v>
       </c>
       <c r="K56" t="n">
-        <v>7.273</v>
+        <v>7.173</v>
       </c>
       <c r="L56" t="n">
-        <v>65.45999999999999</v>
+        <v>64.56</v>
       </c>
       <c r="M56" t="n">
         <v>0</v>
@@ -2770,19 +2770,19 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>1122.082</v>
+        <v>1121.982</v>
       </c>
       <c r="C57" t="n">
-        <v>1122.19</v>
+        <v>1122.09</v>
       </c>
       <c r="D57" t="n">
-        <v>1122.25</v>
+        <v>1122.15</v>
       </c>
       <c r="E57" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="F57" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="G57" t="n">
         <v>9</v>
@@ -2797,10 +2797,10 @@
         <v>355940.049</v>
       </c>
       <c r="K57" t="n">
-        <v>7.232</v>
+        <v>7.132</v>
       </c>
       <c r="L57" t="n">
-        <v>65.09</v>
+        <v>64.19</v>
       </c>
       <c r="M57" t="n">
         <v>0</v>
@@ -2811,19 +2811,19 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>1122.669</v>
+        <v>1122.569</v>
       </c>
       <c r="C58" t="n">
-        <v>1122.25</v>
+        <v>1122.15</v>
       </c>
       <c r="D58" t="n">
-        <v>1123.32</v>
+        <v>1123.22</v>
       </c>
       <c r="E58" t="n">
-        <v>1123.15</v>
+        <v>1123.05</v>
       </c>
       <c r="F58" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="G58" t="n">
         <v>9</v>
@@ -2838,10 +2838,10 @@
         <v>355940.049</v>
       </c>
       <c r="K58" t="n">
-        <v>7.819</v>
+        <v>7.719</v>
       </c>
       <c r="L58" t="n">
-        <v>70.37</v>
+        <v>69.47</v>
       </c>
       <c r="M58" t="n">
         <v>0</v>
@@ -2852,19 +2852,19 @@
         <v>58</v>
       </c>
       <c r="B59" t="n">
-        <v>1125.233</v>
+        <v>1125.133</v>
       </c>
       <c r="C59" t="n">
-        <v>1123.32</v>
+        <v>1123.22</v>
       </c>
       <c r="D59" t="n">
-        <v>1127.12</v>
+        <v>1127.02</v>
       </c>
       <c r="E59" t="n">
-        <v>1127.35</v>
+        <v>1127.25</v>
       </c>
       <c r="F59" t="n">
-        <v>1123.15</v>
+        <v>1123.05</v>
       </c>
       <c r="G59" t="n">
         <v>5.19</v>
@@ -2879,10 +2879,10 @@
         <v>355940.049</v>
       </c>
       <c r="K59" t="n">
-        <v>10.383</v>
+        <v>10.283</v>
       </c>
       <c r="L59" t="n">
-        <v>53.85</v>
+        <v>53.33</v>
       </c>
       <c r="M59" t="n">
         <v>0</v>
@@ -2893,19 +2893,19 @@
         <v>59</v>
       </c>
       <c r="B60" t="n">
-        <v>1122.112</v>
+        <v>1122.012</v>
       </c>
       <c r="C60" t="n">
+        <v>1121.91</v>
+      </c>
+      <c r="D60" t="n">
         <v>1122.01</v>
       </c>
-      <c r="D60" t="n">
-        <v>1122.11</v>
-      </c>
       <c r="E60" t="n">
-        <v>1122.23</v>
+        <v>1122.13</v>
       </c>
       <c r="F60" t="n">
-        <v>1122.11</v>
+        <v>1122.01</v>
       </c>
       <c r="G60" t="n">
         <v>0.08</v>
@@ -2920,7 +2920,7 @@
         <v>355937.049</v>
       </c>
       <c r="K60" t="n">
-        <v>7.262</v>
+        <v>7.162</v>
       </c>
       <c r="L60" t="n">
         <v>0.57</v>
@@ -2934,19 +2934,19 @@
         <v>60</v>
       </c>
       <c r="B61" t="n">
-        <v>1122.21</v>
+        <v>1122.11</v>
       </c>
       <c r="C61" t="n">
+        <v>1122.01</v>
+      </c>
+      <c r="D61" t="n">
         <v>1122.11</v>
       </c>
-      <c r="D61" t="n">
-        <v>1122.21</v>
-      </c>
       <c r="E61" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="F61" t="n">
-        <v>1122.23</v>
+        <v>1122.13</v>
       </c>
       <c r="G61" t="n">
         <v>8.109999999999999</v>
@@ -2961,10 +2961,10 @@
         <v>355937.049</v>
       </c>
       <c r="K61" t="n">
-        <v>7.36</v>
+        <v>7.26</v>
       </c>
       <c r="L61" t="n">
-        <v>59.72</v>
+        <v>58.91</v>
       </c>
       <c r="M61" t="n">
         <v>0</v>
@@ -2975,19 +2975,19 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>1122.051</v>
+        <v>1121.951</v>
       </c>
       <c r="C62" t="n">
-        <v>1122.21</v>
+        <v>1122.11</v>
       </c>
       <c r="D62" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="E62" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="F62" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="G62" t="n">
         <v>9</v>
@@ -3002,10 +3002,10 @@
         <v>355937.049</v>
       </c>
       <c r="K62" t="n">
-        <v>7.201</v>
+        <v>7.101</v>
       </c>
       <c r="L62" t="n">
-        <v>64.81</v>
+        <v>63.91</v>
       </c>
       <c r="M62" t="n">
         <v>0</v>
@@ -3016,19 +3016,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>1121.928</v>
+        <v>1121.828</v>
       </c>
       <c r="C63" t="n">
-        <v>1121.93</v>
+        <v>1121.83</v>
       </c>
       <c r="D63" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="E63" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="F63" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="G63" t="n">
         <v>9</v>
@@ -3043,10 +3043,10 @@
         <v>355937.049</v>
       </c>
       <c r="K63" t="n">
-        <v>7.078</v>
+        <v>6.978</v>
       </c>
       <c r="L63" t="n">
-        <v>63.7</v>
+        <v>62.8</v>
       </c>
       <c r="M63" t="n">
         <v>0</v>
@@ -3057,19 +3057,19 @@
         <v>63</v>
       </c>
       <c r="B64" t="n">
-        <v>1122.554</v>
+        <v>1122.454</v>
       </c>
       <c r="C64" t="n">
-        <v>1121.96</v>
+        <v>1121.86</v>
       </c>
       <c r="D64" t="n">
-        <v>1123.15</v>
+        <v>1123.05</v>
       </c>
       <c r="E64" t="n">
-        <v>1123.06</v>
+        <v>1122.96</v>
       </c>
       <c r="F64" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="G64" t="n">
         <v>9</v>
@@ -3084,10 +3084,10 @@
         <v>355937.049</v>
       </c>
       <c r="K64" t="n">
-        <v>7.704</v>
+        <v>7.604</v>
       </c>
       <c r="L64" t="n">
-        <v>69.33</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="M64" t="n">
         <v>0</v>
@@ -3098,19 +3098,19 @@
         <v>64</v>
       </c>
       <c r="B65" t="n">
-        <v>1124.979</v>
+        <v>1124.879</v>
       </c>
       <c r="C65" t="n">
-        <v>1123.15</v>
+        <v>1123.05</v>
       </c>
       <c r="D65" t="n">
-        <v>1127.35</v>
+        <v>1127.25</v>
       </c>
       <c r="E65" t="n">
-        <v>1126.37</v>
+        <v>1126.27</v>
       </c>
       <c r="F65" t="n">
-        <v>1123.06</v>
+        <v>1122.96</v>
       </c>
       <c r="G65" t="n">
         <v>5.19</v>
@@ -3125,10 +3125,10 @@
         <v>355937.049</v>
       </c>
       <c r="K65" t="n">
-        <v>10.129</v>
+        <v>10.029</v>
       </c>
       <c r="L65" t="n">
-        <v>52.54</v>
+        <v>52.02</v>
       </c>
       <c r="M65" t="n">
         <v>0</v>
@@ -3139,19 +3139,19 @@
         <v>65</v>
       </c>
       <c r="B66" t="n">
-        <v>1122.228</v>
+        <v>1122.128</v>
       </c>
       <c r="C66" t="n">
-        <v>1122.11</v>
+        <v>1122.01</v>
       </c>
       <c r="D66" t="n">
-        <v>1122.23</v>
+        <v>1122.13</v>
       </c>
       <c r="E66" t="n">
-        <v>1122.35</v>
+        <v>1122.25</v>
       </c>
       <c r="F66" t="n">
-        <v>1122.23</v>
+        <v>1122.13</v>
       </c>
       <c r="G66" t="n">
         <v>0.9399999999999999</v>
@@ -3166,10 +3166,10 @@
         <v>355934.049</v>
       </c>
       <c r="K66" t="n">
-        <v>7.378</v>
+        <v>7.278</v>
       </c>
       <c r="L66" t="n">
-        <v>6.96</v>
+        <v>6.86</v>
       </c>
       <c r="M66" t="n">
         <v>0</v>
@@ -3180,19 +3180,19 @@
         <v>66</v>
       </c>
       <c r="B67" t="n">
-        <v>1122.35</v>
+        <v>1122.25</v>
       </c>
       <c r="C67" t="n">
-        <v>1122.23</v>
+        <v>1122.13</v>
       </c>
       <c r="D67" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="E67" t="n">
-        <v>1122.53</v>
+        <v>1122.43</v>
       </c>
       <c r="F67" t="n">
-        <v>1122.35</v>
+        <v>1122.25</v>
       </c>
       <c r="G67" t="n">
         <v>9</v>
@@ -3207,10 +3207,10 @@
         <v>355934.049</v>
       </c>
       <c r="K67" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="L67" t="n">
-        <v>67.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="M67" t="n">
         <v>0</v>
@@ -3221,19 +3221,19 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>1122.221</v>
+        <v>1122.121</v>
       </c>
       <c r="C68" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="D68" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="E68" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="F68" t="n">
-        <v>1122.53</v>
+        <v>1122.43</v>
       </c>
       <c r="G68" t="n">
         <v>9</v>
@@ -3248,10 +3248,10 @@
         <v>355934.049</v>
       </c>
       <c r="K68" t="n">
-        <v>7.371</v>
+        <v>7.271</v>
       </c>
       <c r="L68" t="n">
-        <v>66.34</v>
+        <v>65.44</v>
       </c>
       <c r="M68" t="n">
         <v>0</v>
@@ -3262,19 +3262,19 @@
         <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>1122.097</v>
+        <v>1121.997</v>
       </c>
       <c r="C69" t="n">
-        <v>1121.77</v>
+        <v>1121.67</v>
       </c>
       <c r="D69" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="E69" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="F69" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="G69" t="n">
         <v>9</v>
@@ -3289,10 +3289,10 @@
         <v>355934.049</v>
       </c>
       <c r="K69" t="n">
-        <v>7.247</v>
+        <v>7.147</v>
       </c>
       <c r="L69" t="n">
-        <v>65.22</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="M69" t="n">
         <v>0</v>
@@ -3303,19 +3303,19 @@
         <v>69</v>
       </c>
       <c r="B70" t="n">
-        <v>1122.527</v>
+        <v>1122.427</v>
       </c>
       <c r="C70" t="n">
-        <v>1122.05</v>
+        <v>1121.95</v>
       </c>
       <c r="D70" t="n">
-        <v>1123.06</v>
+        <v>1122.96</v>
       </c>
       <c r="E70" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="F70" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="G70" t="n">
         <v>9</v>
@@ -3330,10 +3330,10 @@
         <v>355934.049</v>
       </c>
       <c r="K70" t="n">
-        <v>7.677</v>
+        <v>7.577</v>
       </c>
       <c r="L70" t="n">
-        <v>69.09999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="M70" t="n">
         <v>0</v>
@@ -3344,19 +3344,19 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>1124.663</v>
+        <v>1124.563</v>
       </c>
       <c r="C71" t="n">
-        <v>1123.06</v>
+        <v>1122.96</v>
       </c>
       <c r="D71" t="n">
-        <v>1126.37</v>
+        <v>1126.27</v>
       </c>
       <c r="E71" t="n">
-        <v>1126.5</v>
+        <v>1126.4</v>
       </c>
       <c r="F71" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="G71" t="n">
         <v>5.19</v>
@@ -3371,10 +3371,10 @@
         <v>355934.049</v>
       </c>
       <c r="K71" t="n">
-        <v>9.813000000000001</v>
+        <v>9.712999999999999</v>
       </c>
       <c r="L71" t="n">
-        <v>50.91</v>
+        <v>50.4</v>
       </c>
       <c r="M71" t="n">
         <v>0</v>
@@ -3385,19 +3385,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="n">
-        <v>1122.34</v>
+        <v>1122.24</v>
       </c>
       <c r="C72" t="n">
-        <v>1122.23</v>
+        <v>1122.13</v>
       </c>
       <c r="D72" t="n">
-        <v>1122.35</v>
+        <v>1122.25</v>
       </c>
       <c r="E72" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="F72" t="n">
-        <v>1122.36</v>
+        <v>1122.26</v>
       </c>
       <c r="G72" t="n">
         <v>0.71</v>
@@ -3412,10 +3412,10 @@
         <v>355931.049</v>
       </c>
       <c r="K72" t="n">
-        <v>7.49</v>
+        <v>7.39</v>
       </c>
       <c r="L72" t="n">
-        <v>5.31</v>
+        <v>5.24</v>
       </c>
       <c r="M72" t="n">
         <v>0</v>
@@ -3426,19 +3426,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>1122.434</v>
+        <v>1122.334</v>
       </c>
       <c r="C73" t="n">
-        <v>1122.35</v>
+        <v>1122.25</v>
       </c>
       <c r="D73" t="n">
-        <v>1122.53</v>
+        <v>1122.43</v>
       </c>
       <c r="E73" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="F73" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="G73" t="n">
         <v>8.23</v>
@@ -3453,10 +3453,10 @@
         <v>355931.049</v>
       </c>
       <c r="K73" t="n">
-        <v>7.584</v>
+        <v>7.484</v>
       </c>
       <c r="L73" t="n">
-        <v>62.4</v>
+        <v>61.58</v>
       </c>
       <c r="M73" t="n">
         <v>0</v>
@@ -3467,19 +3467,19 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>1122.454</v>
+        <v>1122.354</v>
       </c>
       <c r="C74" t="n">
-        <v>1122.53</v>
+        <v>1122.43</v>
       </c>
       <c r="D74" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="E74" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="F74" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="G74" t="n">
         <v>9</v>
@@ -3494,10 +3494,10 @@
         <v>355931.049</v>
       </c>
       <c r="K74" t="n">
-        <v>7.604</v>
+        <v>7.504</v>
       </c>
       <c r="L74" t="n">
-        <v>68.44</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M74" t="n">
         <v>0</v>
@@ -3508,19 +3508,19 @@
         <v>74</v>
       </c>
       <c r="B75" t="n">
-        <v>1122.425</v>
+        <v>1122.325</v>
       </c>
       <c r="C75" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="D75" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="E75" t="n">
-        <v>1122.58</v>
+        <v>1122.48</v>
       </c>
       <c r="F75" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="G75" t="n">
         <v>9</v>
@@ -3535,10 +3535,10 @@
         <v>355931.049</v>
       </c>
       <c r="K75" t="n">
-        <v>7.575</v>
+        <v>7.475</v>
       </c>
       <c r="L75" t="n">
-        <v>68.18000000000001</v>
+        <v>67.28</v>
       </c>
       <c r="M75" t="n">
         <v>0</v>
@@ -3549,19 +3549,19 @@
         <v>75</v>
       </c>
       <c r="B76" t="n">
-        <v>1122.75</v>
+        <v>1122.65</v>
       </c>
       <c r="C76" t="n">
-        <v>1122.27</v>
+        <v>1122.17</v>
       </c>
       <c r="D76" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="E76" t="n">
-        <v>1123.42</v>
+        <v>1123.32</v>
       </c>
       <c r="F76" t="n">
-        <v>1122.58</v>
+        <v>1122.48</v>
       </c>
       <c r="G76" t="n">
         <v>9</v>
@@ -3576,10 +3576,10 @@
         <v>355931.049</v>
       </c>
       <c r="K76" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="L76" t="n">
-        <v>71.09999999999999</v>
+        <v>70.2</v>
       </c>
       <c r="M76" t="n">
         <v>0</v>
@@ -3590,19 +3590,19 @@
         <v>76</v>
       </c>
       <c r="B77" t="n">
-        <v>1124.73</v>
+        <v>1124.63</v>
       </c>
       <c r="C77" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="D77" t="n">
-        <v>1126.5</v>
+        <v>1126.4</v>
       </c>
       <c r="E77" t="n">
-        <v>1126.27</v>
+        <v>1126.17</v>
       </c>
       <c r="F77" t="n">
-        <v>1123.42</v>
+        <v>1123.32</v>
       </c>
       <c r="G77" t="n">
         <v>5.19</v>
@@ -3617,10 +3617,10 @@
         <v>355931.049</v>
       </c>
       <c r="K77" t="n">
-        <v>9.880000000000001</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="L77" t="n">
-        <v>51.28</v>
+        <v>50.76</v>
       </c>
       <c r="M77" t="n">
         <v>0</v>
@@ -3631,19 +3631,19 @@
         <v>77</v>
       </c>
       <c r="B78" t="n">
-        <v>1122.413</v>
+        <v>1122.313</v>
       </c>
       <c r="C78" t="n">
-        <v>1122.36</v>
+        <v>1122.26</v>
       </c>
       <c r="D78" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="E78" t="n">
-        <v>1122.48</v>
+        <v>1122.38</v>
       </c>
       <c r="F78" t="n">
-        <v>1122.39</v>
+        <v>1122.29</v>
       </c>
       <c r="G78" t="n">
         <v>0.1</v>
@@ -3658,10 +3658,10 @@
         <v>355928.049</v>
       </c>
       <c r="K78" t="n">
-        <v>7.563</v>
+        <v>7.463</v>
       </c>
       <c r="L78" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="M78" t="n">
         <v>0</v>
@@ -3672,19 +3672,19 @@
         <v>78</v>
       </c>
       <c r="B79" t="n">
-        <v>1122.458</v>
+        <v>1122.358</v>
       </c>
       <c r="C79" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="D79" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="E79" t="n">
-        <v>1122.5</v>
+        <v>1122.4</v>
       </c>
       <c r="F79" t="n">
-        <v>1122.48</v>
+        <v>1122.38</v>
       </c>
       <c r="G79" t="n">
         <v>8.449999999999999</v>
@@ -3699,10 +3699,10 @@
         <v>355928.049</v>
       </c>
       <c r="K79" t="n">
-        <v>7.608</v>
+        <v>7.508</v>
       </c>
       <c r="L79" t="n">
-        <v>64.31</v>
+        <v>63.47</v>
       </c>
       <c r="M79" t="n">
         <v>0</v>
@@ -3713,19 +3713,19 @@
         <v>79</v>
       </c>
       <c r="B80" t="n">
-        <v>1122.496</v>
+        <v>1122.396</v>
       </c>
       <c r="C80" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="D80" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="E80" t="n">
-        <v>1122.49</v>
+        <v>1122.39</v>
       </c>
       <c r="F80" t="n">
-        <v>1122.5</v>
+        <v>1122.4</v>
       </c>
       <c r="G80" t="n">
         <v>9</v>
@@ -3740,10 +3740,10 @@
         <v>355928.049</v>
       </c>
       <c r="K80" t="n">
-        <v>7.646</v>
+        <v>7.546</v>
       </c>
       <c r="L80" t="n">
-        <v>68.81</v>
+        <v>67.91</v>
       </c>
       <c r="M80" t="n">
         <v>0</v>
@@ -3754,19 +3754,19 @@
         <v>80</v>
       </c>
       <c r="B81" t="n">
-        <v>1122.9</v>
+        <v>1122.8</v>
       </c>
       <c r="C81" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="D81" t="n">
-        <v>1122.58</v>
+        <v>1122.48</v>
       </c>
       <c r="E81" t="n">
-        <v>1123.97</v>
+        <v>1123.87</v>
       </c>
       <c r="F81" t="n">
-        <v>1122.49</v>
+        <v>1122.39</v>
       </c>
       <c r="G81" t="n">
         <v>9</v>
@@ -3781,10 +3781,10 @@
         <v>355928.049</v>
       </c>
       <c r="K81" t="n">
-        <v>8.050000000000001</v>
+        <v>7.95</v>
       </c>
       <c r="L81" t="n">
-        <v>72.45</v>
+        <v>71.55</v>
       </c>
       <c r="M81" t="n">
         <v>0</v>
@@ -3795,19 +3795,19 @@
         <v>81</v>
       </c>
       <c r="B82" t="n">
-        <v>1123.878</v>
+        <v>1123.778</v>
       </c>
       <c r="C82" t="n">
-        <v>1122.58</v>
+        <v>1122.48</v>
       </c>
       <c r="D82" t="n">
-        <v>1123.42</v>
+        <v>1123.32</v>
       </c>
       <c r="E82" t="n">
-        <v>1125.55</v>
+        <v>1125.45</v>
       </c>
       <c r="F82" t="n">
-        <v>1123.97</v>
+        <v>1123.87</v>
       </c>
       <c r="G82" t="n">
         <v>9</v>
@@ -3822,10 +3822,10 @@
         <v>355928.049</v>
       </c>
       <c r="K82" t="n">
-        <v>9.028</v>
+        <v>8.928000000000001</v>
       </c>
       <c r="L82" t="n">
-        <v>81.26000000000001</v>
+        <v>80.36</v>
       </c>
       <c r="M82" t="n">
         <v>0</v>
@@ -3836,19 +3836,19 @@
         <v>82</v>
       </c>
       <c r="B83" t="n">
-        <v>1125.522</v>
+        <v>1125.422</v>
       </c>
       <c r="C83" t="n">
-        <v>1123.42</v>
+        <v>1123.32</v>
       </c>
       <c r="D83" t="n">
-        <v>1126.27</v>
+        <v>1126.17</v>
       </c>
       <c r="E83" t="n">
-        <v>1126.85</v>
+        <v>1126.75</v>
       </c>
       <c r="F83" t="n">
-        <v>1125.55</v>
+        <v>1125.45</v>
       </c>
       <c r="G83" t="n">
         <v>5.19</v>
@@ -3863,10 +3863,10 @@
         <v>355928.049</v>
       </c>
       <c r="K83" t="n">
-        <v>10.672</v>
+        <v>10.572</v>
       </c>
       <c r="L83" t="n">
-        <v>55.4</v>
+        <v>54.88</v>
       </c>
       <c r="M83" t="n">
         <v>0</v>
@@ -3877,19 +3877,19 @@
         <v>83</v>
       </c>
       <c r="B84" t="n">
-        <v>1122.307</v>
+        <v>1122.207</v>
       </c>
       <c r="C84" t="n">
-        <v>1122.39</v>
+        <v>1122.29</v>
       </c>
       <c r="D84" t="n">
-        <v>1122.39</v>
+        <v>1122.29</v>
       </c>
       <c r="E84" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="F84" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="G84" t="n">
         <v>0.11</v>
@@ -3904,10 +3904,10 @@
         <v>355925.049</v>
       </c>
       <c r="K84" t="n">
-        <v>7.457</v>
+        <v>7.357</v>
       </c>
       <c r="L84" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="M84" t="n">
         <v>0</v>
@@ -3918,19 +3918,19 @@
         <v>84</v>
       </c>
       <c r="B85" t="n">
-        <v>1122.398</v>
+        <v>1122.298</v>
       </c>
       <c r="C85" t="n">
-        <v>1122.39</v>
+        <v>1122.29</v>
       </c>
       <c r="D85" t="n">
-        <v>1122.48</v>
+        <v>1122.38</v>
       </c>
       <c r="E85" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="F85" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="G85" t="n">
         <v>3.74</v>
@@ -3945,10 +3945,10 @@
         <v>355925.049</v>
       </c>
       <c r="K85" t="n">
-        <v>7.548</v>
+        <v>7.448</v>
       </c>
       <c r="L85" t="n">
-        <v>28.24</v>
+        <v>27.87</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3959,19 +3959,19 @@
         <v>85</v>
       </c>
       <c r="B86" t="n">
-        <v>1122.491</v>
+        <v>1122.391</v>
       </c>
       <c r="C86" t="n">
-        <v>1122.48</v>
+        <v>1122.38</v>
       </c>
       <c r="D86" t="n">
-        <v>1122.5</v>
+        <v>1122.4</v>
       </c>
       <c r="E86" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="F86" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="G86" t="n">
         <v>9</v>
@@ -3986,10 +3986,10 @@
         <v>355925.049</v>
       </c>
       <c r="K86" t="n">
-        <v>7.641</v>
+        <v>7.541</v>
       </c>
       <c r="L86" t="n">
-        <v>68.77</v>
+        <v>67.87</v>
       </c>
       <c r="M86" t="n">
         <v>0</v>
@@ -4000,19 +4000,19 @@
         <v>86</v>
       </c>
       <c r="B87" t="n">
-        <v>1122.707</v>
+        <v>1122.607</v>
       </c>
       <c r="C87" t="n">
-        <v>1122.5</v>
+        <v>1122.4</v>
       </c>
       <c r="D87" t="n">
-        <v>1122.49</v>
+        <v>1122.39</v>
       </c>
       <c r="E87" t="n">
-        <v>1123.28</v>
+        <v>1123.18</v>
       </c>
       <c r="F87" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="G87" t="n">
         <v>9</v>
@@ -4027,10 +4027,10 @@
         <v>355925.049</v>
       </c>
       <c r="K87" t="n">
-        <v>7.857</v>
+        <v>7.757</v>
       </c>
       <c r="L87" t="n">
-        <v>70.70999999999999</v>
+        <v>69.81</v>
       </c>
       <c r="M87" t="n">
         <v>0</v>
@@ -4041,19 +4041,19 @@
         <v>87</v>
       </c>
       <c r="B88" t="n">
-        <v>1123.623</v>
+        <v>1123.523</v>
       </c>
       <c r="C88" t="n">
-        <v>1122.49</v>
+        <v>1122.39</v>
       </c>
       <c r="D88" t="n">
-        <v>1123.97</v>
+        <v>1123.87</v>
       </c>
       <c r="E88" t="n">
-        <v>1124.75</v>
+        <v>1124.65</v>
       </c>
       <c r="F88" t="n">
-        <v>1123.28</v>
+        <v>1123.18</v>
       </c>
       <c r="G88" t="n">
         <v>9</v>
@@ -4068,10 +4068,10 @@
         <v>355925.049</v>
       </c>
       <c r="K88" t="n">
-        <v>8.773</v>
+        <v>8.673</v>
       </c>
       <c r="L88" t="n">
-        <v>78.95999999999999</v>
+        <v>78.06</v>
       </c>
       <c r="M88" t="n">
         <v>0</v>
@@ -4082,19 +4082,19 @@
         <v>88</v>
       </c>
       <c r="B89" t="n">
-        <v>1125.023</v>
+        <v>1124.923</v>
       </c>
       <c r="C89" t="n">
-        <v>1123.97</v>
+        <v>1123.87</v>
       </c>
       <c r="D89" t="n">
-        <v>1125.55</v>
+        <v>1125.45</v>
       </c>
       <c r="E89" t="n">
-        <v>1125.82</v>
+        <v>1125.72</v>
       </c>
       <c r="F89" t="n">
-        <v>1124.75</v>
+        <v>1124.65</v>
       </c>
       <c r="G89" t="n">
         <v>9</v>
@@ -4109,10 +4109,10 @@
         <v>355925.049</v>
       </c>
       <c r="K89" t="n">
-        <v>10.173</v>
+        <v>10.073</v>
       </c>
       <c r="L89" t="n">
-        <v>91.55</v>
+        <v>90.65000000000001</v>
       </c>
       <c r="M89" t="n">
         <v>0</v>
@@ -4123,19 +4123,19 @@
         <v>89</v>
       </c>
       <c r="B90" t="n">
-        <v>1126.219</v>
+        <v>1126.119</v>
       </c>
       <c r="C90" t="n">
-        <v>1125.55</v>
+        <v>1125.45</v>
       </c>
       <c r="D90" t="n">
-        <v>1126.85</v>
+        <v>1126.75</v>
       </c>
       <c r="E90" t="n">
-        <v>1126.66</v>
+        <v>1126.56</v>
       </c>
       <c r="F90" t="n">
-        <v>1125.82</v>
+        <v>1125.72</v>
       </c>
       <c r="G90" t="n">
         <v>5.17</v>
@@ -4150,10 +4150,10 @@
         <v>355925.049</v>
       </c>
       <c r="K90" t="n">
-        <v>11.369</v>
+        <v>11.269</v>
       </c>
       <c r="L90" t="n">
-        <v>58.79</v>
+        <v>58.27</v>
       </c>
       <c r="M90" t="n">
         <v>0</v>
@@ -4164,19 +4164,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="n">
-        <v>1122.285</v>
+        <v>1122.185</v>
       </c>
       <c r="C91" t="n">
-        <v>1122.15</v>
+        <v>1122.05</v>
       </c>
       <c r="D91" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="E91" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="F91" t="n">
-        <v>1122.28</v>
+        <v>1122.18</v>
       </c>
       <c r="G91" t="n">
         <v>1.03</v>
@@ -4191,10 +4191,10 @@
         <v>355922.049</v>
       </c>
       <c r="K91" t="n">
-        <v>7.435</v>
+        <v>7.335</v>
       </c>
       <c r="L91" t="n">
-        <v>7.69</v>
+        <v>7.59</v>
       </c>
       <c r="M91" t="n">
         <v>0</v>
@@ -4205,19 +4205,19 @@
         <v>91</v>
       </c>
       <c r="B92" t="n">
-        <v>1122.425</v>
+        <v>1122.325</v>
       </c>
       <c r="C92" t="n">
-        <v>1122.29</v>
+        <v>1122.19</v>
       </c>
       <c r="D92" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="E92" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="F92" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="G92" t="n">
         <v>9</v>
@@ -4232,10 +4232,10 @@
         <v>355922.049</v>
       </c>
       <c r="K92" t="n">
-        <v>7.575</v>
+        <v>7.475</v>
       </c>
       <c r="L92" t="n">
-        <v>68.17</v>
+        <v>67.27</v>
       </c>
       <c r="M92" t="n">
         <v>0</v>
@@ -4246,19 +4246,19 @@
         <v>92</v>
       </c>
       <c r="B93" t="n">
-        <v>1122.547</v>
+        <v>1122.447</v>
       </c>
       <c r="C93" t="n">
-        <v>1122.43</v>
+        <v>1122.33</v>
       </c>
       <c r="D93" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="E93" t="n">
-        <v>1122.64</v>
+        <v>1122.54</v>
       </c>
       <c r="F93" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="G93" t="n">
         <v>9</v>
@@ -4273,10 +4273,10 @@
         <v>355922.049</v>
       </c>
       <c r="K93" t="n">
-        <v>7.697</v>
+        <v>7.597</v>
       </c>
       <c r="L93" t="n">
-        <v>69.28</v>
+        <v>68.38</v>
       </c>
       <c r="M93" t="n">
         <v>0</v>
@@ -4287,19 +4287,19 @@
         <v>93</v>
       </c>
       <c r="B94" t="n">
-        <v>1122.99</v>
+        <v>1122.89</v>
       </c>
       <c r="C94" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="D94" t="n">
-        <v>1123.28</v>
+        <v>1123.18</v>
       </c>
       <c r="E94" t="n">
-        <v>1123.48</v>
+        <v>1123.38</v>
       </c>
       <c r="F94" t="n">
-        <v>1122.64</v>
+        <v>1122.54</v>
       </c>
       <c r="G94" t="n">
         <v>9</v>
@@ -4314,10 +4314,10 @@
         <v>355922.049</v>
       </c>
       <c r="K94" t="n">
-        <v>8.140000000000001</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="L94" t="n">
-        <v>73.26000000000001</v>
+        <v>72.36</v>
       </c>
       <c r="M94" t="n">
         <v>0</v>
@@ -4328,19 +4328,19 @@
         <v>94</v>
       </c>
       <c r="B95" t="n">
-        <v>1124.022</v>
+        <v>1123.922</v>
       </c>
       <c r="C95" t="n">
-        <v>1123.28</v>
+        <v>1123.18</v>
       </c>
       <c r="D95" t="n">
-        <v>1124.75</v>
+        <v>1124.65</v>
       </c>
       <c r="E95" t="n">
-        <v>1124.58</v>
+        <v>1124.48</v>
       </c>
       <c r="F95" t="n">
-        <v>1123.48</v>
+        <v>1123.38</v>
       </c>
       <c r="G95" t="n">
         <v>9</v>
@@ -4355,10 +4355,10 @@
         <v>355922.049</v>
       </c>
       <c r="K95" t="n">
-        <v>9.172000000000001</v>
+        <v>9.071999999999999</v>
       </c>
       <c r="L95" t="n">
-        <v>82.55</v>
+        <v>81.65000000000001</v>
       </c>
       <c r="M95" t="n">
         <v>0</v>
@@ -4369,19 +4369,19 @@
         <v>95</v>
       </c>
       <c r="B96" t="n">
-        <v>1125.382</v>
+        <v>1125.282</v>
       </c>
       <c r="C96" t="n">
-        <v>1124.75</v>
+        <v>1124.65</v>
       </c>
       <c r="D96" t="n">
-        <v>1125.82</v>
+        <v>1125.72</v>
       </c>
       <c r="E96" t="n">
-        <v>1126.38</v>
+        <v>1126.28</v>
       </c>
       <c r="F96" t="n">
-        <v>1124.58</v>
+        <v>1124.48</v>
       </c>
       <c r="G96" t="n">
         <v>9</v>
@@ -4396,10 +4396,10 @@
         <v>355922.049</v>
       </c>
       <c r="K96" t="n">
-        <v>10.532</v>
+        <v>10.432</v>
       </c>
       <c r="L96" t="n">
-        <v>94.78</v>
+        <v>93.88</v>
       </c>
       <c r="M96" t="n">
         <v>0</v>
@@ -4410,19 +4410,19 @@
         <v>96</v>
       </c>
       <c r="B97" t="n">
-        <v>1126.321</v>
+        <v>1126.221</v>
       </c>
       <c r="C97" t="n">
-        <v>1125.82</v>
+        <v>1125.72</v>
       </c>
       <c r="D97" t="n">
-        <v>1126.66</v>
+        <v>1126.56</v>
       </c>
       <c r="E97" t="n">
-        <v>1126.43</v>
+        <v>1126.33</v>
       </c>
       <c r="F97" t="n">
-        <v>1126.38</v>
+        <v>1126.28</v>
       </c>
       <c r="G97" t="n">
         <v>3.69</v>
@@ -4437,10 +4437,10 @@
         <v>355922.049</v>
       </c>
       <c r="K97" t="n">
-        <v>11.471</v>
+        <v>11.371</v>
       </c>
       <c r="L97" t="n">
-        <v>42.32</v>
+        <v>41.95</v>
       </c>
       <c r="M97" t="n">
         <v>0</v>
@@ -4451,19 +4451,19 @@
         <v>97</v>
       </c>
       <c r="B98" t="n">
-        <v>1122.436</v>
+        <v>1122.336</v>
       </c>
       <c r="C98" t="n">
-        <v>1122.28</v>
+        <v>1122.18</v>
       </c>
       <c r="D98" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="E98" t="n">
-        <v>1122.6</v>
+        <v>1122.5</v>
       </c>
       <c r="F98" t="n">
-        <v>1122.46</v>
+        <v>1122.36</v>
       </c>
       <c r="G98" t="n">
         <v>2.31</v>
@@ -4478,10 +4478,10 @@
         <v>355919.049</v>
       </c>
       <c r="K98" t="n">
-        <v>7.586</v>
+        <v>7.486</v>
       </c>
       <c r="L98" t="n">
-        <v>17.52</v>
+        <v>17.29</v>
       </c>
       <c r="M98" t="n">
         <v>0</v>
@@ -4492,19 +4492,19 @@
         <v>98</v>
       </c>
       <c r="B99" t="n">
-        <v>1122.575</v>
+        <v>1122.475</v>
       </c>
       <c r="C99" t="n">
-        <v>1122.42</v>
+        <v>1122.32</v>
       </c>
       <c r="D99" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="E99" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="F99" t="n">
-        <v>1122.6</v>
+        <v>1122.5</v>
       </c>
       <c r="G99" t="n">
         <v>8.44</v>
@@ -4519,10 +4519,10 @@
         <v>355919.049</v>
       </c>
       <c r="K99" t="n">
-        <v>7.725</v>
+        <v>7.625</v>
       </c>
       <c r="L99" t="n">
-        <v>65.2</v>
+        <v>64.36</v>
       </c>
       <c r="M99" t="n">
         <v>0</v>
@@ -4533,19 +4533,19 @@
         <v>99</v>
       </c>
       <c r="B100" t="n">
-        <v>1122.672</v>
+        <v>1122.572</v>
       </c>
       <c r="C100" t="n">
-        <v>1122.56</v>
+        <v>1122.46</v>
       </c>
       <c r="D100" t="n">
-        <v>1122.64</v>
+        <v>1122.54</v>
       </c>
       <c r="E100" t="n">
-        <v>1122.76</v>
+        <v>1122.66</v>
       </c>
       <c r="F100" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="G100" t="n">
         <v>7.52</v>
@@ -4560,10 +4560,10 @@
         <v>355919.049</v>
       </c>
       <c r="K100" t="n">
-        <v>7.822</v>
+        <v>7.722</v>
       </c>
       <c r="L100" t="n">
-        <v>58.84</v>
+        <v>58.09</v>
       </c>
       <c r="M100" t="n">
         <v>0</v>
@@ -4574,19 +4574,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="n">
-        <v>1122.962</v>
+        <v>1122.862</v>
       </c>
       <c r="C101" t="n">
-        <v>1122.64</v>
+        <v>1122.54</v>
       </c>
       <c r="D101" t="n">
-        <v>1123.48</v>
+        <v>1123.38</v>
       </c>
       <c r="E101" t="n">
-        <v>1122.97</v>
+        <v>1122.87</v>
       </c>
       <c r="F101" t="n">
-        <v>1122.76</v>
+        <v>1122.66</v>
       </c>
       <c r="G101" t="n">
         <v>8.58</v>
@@ -4601,10 +4601,10 @@
         <v>355919.049</v>
       </c>
       <c r="K101" t="n">
-        <v>8.112</v>
+        <v>8.012</v>
       </c>
       <c r="L101" t="n">
-        <v>69.61</v>
+        <v>68.75</v>
       </c>
       <c r="M101" t="n">
         <v>0</v>
@@ -4615,19 +4615,19 @@
         <v>101</v>
       </c>
       <c r="B102" t="n">
-        <v>1123.811</v>
+        <v>1123.711</v>
       </c>
       <c r="C102" t="n">
-        <v>1123.48</v>
+        <v>1123.38</v>
       </c>
       <c r="D102" t="n">
-        <v>1124.58</v>
+        <v>1124.48</v>
       </c>
       <c r="E102" t="n">
-        <v>1124.22</v>
+        <v>1124.12</v>
       </c>
       <c r="F102" t="n">
-        <v>1122.97</v>
+        <v>1122.87</v>
       </c>
       <c r="G102" t="n">
         <v>8.84</v>
@@ -4642,10 +4642,10 @@
         <v>355919.049</v>
       </c>
       <c r="K102" t="n">
-        <v>8.961</v>
+        <v>8.861000000000001</v>
       </c>
       <c r="L102" t="n">
-        <v>79.2</v>
+        <v>78.31</v>
       </c>
       <c r="M102" t="n">
         <v>0</v>
@@ -4656,19 +4656,19 @@
         <v>102</v>
       </c>
       <c r="B103" t="n">
-        <v>1125.276</v>
+        <v>1125.176</v>
       </c>
       <c r="C103" t="n">
-        <v>1124.58</v>
+        <v>1124.48</v>
       </c>
       <c r="D103" t="n">
-        <v>1126.38</v>
+        <v>1126.28</v>
       </c>
       <c r="E103" t="n">
-        <v>1125.93</v>
+        <v>1125.83</v>
       </c>
       <c r="F103" t="n">
-        <v>1124.22</v>
+        <v>1124.12</v>
       </c>
       <c r="G103" t="n">
         <v>5.65</v>
@@ -4683,10 +4683,10 @@
         <v>355919.049</v>
       </c>
       <c r="K103" t="n">
-        <v>10.426</v>
+        <v>10.326</v>
       </c>
       <c r="L103" t="n">
-        <v>58.86</v>
+        <v>58.29</v>
       </c>
       <c r="M103" t="n">
         <v>0</v>
@@ -4697,19 +4697,19 @@
         <v>103</v>
       </c>
       <c r="B104" t="n">
-        <v>1126.288</v>
+        <v>1126.188</v>
       </c>
       <c r="C104" t="n">
-        <v>1126.38</v>
+        <v>1126.28</v>
       </c>
       <c r="D104" t="n">
-        <v>1126.43</v>
+        <v>1126.33</v>
       </c>
       <c r="E104" t="n">
-        <v>1126.41</v>
+        <v>1126.31</v>
       </c>
       <c r="F104" t="n">
-        <v>1125.93</v>
+        <v>1125.83</v>
       </c>
       <c r="G104" t="n">
         <v>0.19</v>
@@ -4724,10 +4724,10 @@
         <v>355919.049</v>
       </c>
       <c r="K104" t="n">
-        <v>11.438</v>
+        <v>11.338</v>
       </c>
       <c r="L104" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="M104" t="n">
         <v>0</v>
@@ -4738,19 +4738,19 @@
         <v>104</v>
       </c>
       <c r="B105" t="n">
-        <v>1122.599</v>
+        <v>1122.499</v>
       </c>
       <c r="C105" t="n">
-        <v>1122.46</v>
+        <v>1122.36</v>
       </c>
       <c r="D105" t="n">
-        <v>1122.6</v>
+        <v>1122.5</v>
       </c>
       <c r="E105" t="n">
-        <v>1122.78</v>
+        <v>1122.68</v>
       </c>
       <c r="F105" t="n">
-        <v>1122.57</v>
+        <v>1122.47</v>
       </c>
       <c r="G105" t="n">
         <v>0.5</v>
@@ -4765,10 +4765,10 @@
         <v>355916.049</v>
       </c>
       <c r="K105" t="n">
-        <v>7.749</v>
+        <v>7.649</v>
       </c>
       <c r="L105" t="n">
-        <v>3.9</v>
+        <v>3.85</v>
       </c>
       <c r="M105" t="n">
         <v>0</v>
@@ -4779,19 +4779,19 @@
         <v>105</v>
       </c>
       <c r="B106" t="n">
-        <v>1122.747</v>
+        <v>1122.647</v>
       </c>
       <c r="C106" t="n">
-        <v>1122.6</v>
+        <v>1122.5</v>
       </c>
       <c r="D106" t="n">
-        <v>1122.73</v>
+        <v>1122.63</v>
       </c>
       <c r="E106" t="n">
-        <v>1122.89</v>
+        <v>1122.79</v>
       </c>
       <c r="F106" t="n">
-        <v>1122.78</v>
+        <v>1122.68</v>
       </c>
       <c r="G106" t="n">
         <v>1.41</v>
@@ -4806,10 +4806,10 @@
         <v>355916.049</v>
       </c>
       <c r="K106" t="n">
-        <v>7.897</v>
+        <v>7.797</v>
       </c>
       <c r="L106" t="n">
-        <v>11.11</v>
+        <v>10.97</v>
       </c>
       <c r="M106" t="n">
         <v>0</v>
@@ -4820,19 +4820,19 @@
         <v>106</v>
       </c>
       <c r="B107" t="n">
-        <v>1123.92</v>
+        <v>1123.82</v>
       </c>
       <c r="C107" t="n">
-        <v>1122.97</v>
+        <v>1122.87</v>
       </c>
       <c r="D107" t="n">
-        <v>1124.22</v>
+        <v>1124.12</v>
       </c>
       <c r="E107" t="n">
-        <v>1124.8</v>
+        <v>1124.7</v>
       </c>
       <c r="F107" t="n">
-        <v>1123.69</v>
+        <v>1123.59</v>
       </c>
       <c r="G107" t="n">
         <v>0.1</v>
@@ -4847,10 +4847,10 @@
         <v>355916.049</v>
       </c>
       <c r="K107" t="n">
-        <v>9.07</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="L107" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="M107" t="n">
         <v>0</v>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>all ground levels lowered by 0.15</t>
+          <t>all ground levels lowered by 0.25</t>
         </is>
       </c>
     </row>
@@ -4915,7 +4915,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>5354.85</v>
+        <v>5288.33</v>
       </c>
     </row>
     <row r="115">
@@ -4935,7 +4935,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1122.901</v>
+        <v>1122.801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>